<commit_message>
Chore: Updated README.md and added additional sample_data
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -26,7 +26,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -35,12 +35,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,10 +61,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,181 +464,166 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AP3</t>
+          <t>AP36</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP3, Frequency=774, Hop_Value=0xB7</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP36, Frequency=780, Hop_Value=0x98</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP3, Frequency=775, Hop_Value=0xB7</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>frequency</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP36, Frequency=780, Hop_Value=0x98</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AP9</t>
+          <t>AP47</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISSING_FILE2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP9, Frequency=765, Hop_Value=0x49</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP9, Frequency=765, Hop_Value=0x49</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP47, Frequency=775, Hop_Value=0x1A</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AP2</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+          <t>AP1</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP2, Frequency=784, Hop_Value=0x19</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP1, Frequency=777, Hop_Value=0xE2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP2, Frequency=784, Hop_Value=0x19</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP1, Frequency=777, Hop_Value=0xE2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AP32</t>
+          <t>AP50</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISSING_FILE2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP32, Frequency=769, Hop_Value=0x68</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP32, Frequency=769, Hop_Value=0x68</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP50, Frequency=763, Hop_Value=0x8C</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AP44</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+          <t>AP27</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP44, Frequency=790, Hop_Value=0x56</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP27, Frequency=762, Hop_Value=0x9E</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP44, Frequency=790, Hop_Value=0x56</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP27, Frequency=762, Hop_Value=0x9E</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AP10</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP7</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP10, Frequency=768, Hop_Value=0x17</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP7, Frequency=767, Hop_Value=0xE9</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP10, Frequency=768, Hop_Value=0x17</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP7, Frequency=767, Hop_Value=0xAA</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AP49</t>
+          <t>AP54</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>MATCH</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP49, Frequency=774, Hop_Value=0x3F</t>
+          <t>MISSING_FILE1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP49, Frequency=774, Hop_Value=0x3F</t>
+          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP54, Frequency=785, Hop_Value=0x78</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AP15</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
+          <t>AP2</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>MISMATCH</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP15, Frequency=781, Hop_Value=0x7E</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP2, Frequency=784, Hop_Value=0x19</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP15, Frequency=782, Hop_Value=0x7E</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP2, Frequency=785, Hop_Value=0x19</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -644,954 +635,1049 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AP22</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP44</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP22, Frequency=772, Hop_Value=0x33</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP44, Frequency=790, Hop_Value=0x56</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP22, Frequency=772, Hop_Value=0x33</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP44, Frequency=790, Hop_Value=0x57</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AP46</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
+          <t>AP39</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP46, Frequency=786, Hop_Value=0x79</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP39, Frequency=767, Hop_Value=0x6A</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP46, Frequency=786, Hop_Value=0x79</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP39, Frequency=767, Hop_Value=0x6A</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AP30</t>
+          <t>AP32</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP30, Frequency=776, Hop_Value=0xA0</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP32, Frequency=769, Hop_Value=0x68</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP30, Frequency=776, Hop_Value=0xA1</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>frequency_hop_value</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP32, Frequency=769, Hop_Value=0x68</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AP24</t>
+          <t>AP52</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>MATCH</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP24, Frequency=768, Hop_Value=0xC6</t>
+          <t>MISSING_FILE1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP24, Frequency=768, Hop_Value=0xC6</t>
+          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP52, Frequency=783, Hop_Value=0x34</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AP26</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
+          <t>AP14</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP26, Frequency=785, Hop_Value=0xBB</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP14, Frequency=777, Hop_Value=0xCC</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP26, Frequency=785, Hop_Value=0xBB</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP14, Frequency=777, Hop_Value=0xCC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AP45</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
+          <t>AP19</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP45, Frequency=764, Hop_Value=0xA5</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP19, Frequency=777, Hop_Value=0xE9</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP45, Frequency=764, Hop_Value=0xA5</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP19, Frequency=777, Hop_Value=0xE9</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AP12</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
+          <t>AP5</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP12, Frequency=784, Hop_Value=0x30</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP5, Frequency=781, Hop_Value=0x6D</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP12, Frequency=784, Hop_Value=0x30</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP5, Frequency=781, Hop_Value=0x6D</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AP6</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
+          <t>AP3</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP6, Frequency=784, Hop_Value=0x8E</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP3, Frequency=774, Hop_Value=0xB7</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP6, Frequency=784, Hop_Value=0x8E</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP3, Frequency=774, Hop_Value=0xB7</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AP35</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
+          <t>AP11</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP35, Frequency=784, Hop_Value=0x36</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP11, Frequency=766, Hop_Value=0xEF</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP35, Frequency=784, Hop_Value=0x36</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP11, Frequency=766, Hop_Value=0xEF</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AP18</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
+          <t>AP45</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP18, Frequency=764, Hop_Value=0x1D</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP45, Frequency=764, Hop_Value=0xA5</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP18, Frequency=764, Hop_Value=0x1D</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP45, Frequency=764, Hop_Value=0xA5</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AP29</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP18</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP29, Frequency=776, Hop_Value=0x3A</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP18, Frequency=764, Hop_Value=0x1D</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP29, Frequency=776, Hop_Value=0x3A</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP18, Frequency=764, Hop_Value=0x2D</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AP5</t>
-        </is>
-      </c>
-      <c r="B21" s="1" t="inlineStr">
+          <t>AP12</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>MISMATCH</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP5, Frequency=781, Hop_Value=0x6D</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP12, Frequency=784, Hop_Value=0x30</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP5, Frequency=780, Hop_Value=0x6D</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP12, Frequency=784, Hop_Value=0x31</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>frequency</t>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AP50</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
+          <t>AP28</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP50, Frequency=763, Hop_Value=0x8C</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP28, Frequency=781, Hop_Value=0x46</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP50, Frequency=763, Hop_Value=0x8C</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP28, Frequency=781, Hop_Value=0x46</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AP19</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
+          <t>AP41</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP19, Frequency=777, Hop_Value=0xE9</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP41, Frequency=776, Hop_Value=0xA5</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP19, Frequency=777, Hop_Value=0xE9</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP41, Frequency=776, Hop_Value=0xA5</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AP11</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+          <t>AP37</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>MISMATCH</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP11, Frequency=766, Hop_Value=0xEF</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP37, Frequency=773, Hop_Value=0xC3</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP11, Frequency=766, Hop_Value=0xEE</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP37, Frequency=774, Hop_Value=0xC3</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>frequency_hop_value</t>
+          <t>frequency</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AP28</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
+          <t>AP9</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP28, Frequency=781, Hop_Value=0x46</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP9, Frequency=765, Hop_Value=0x49</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP28, Frequency=781, Hop_Value=0x46</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP9, Frequency=765, Hop_Value=0x49</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AP34</t>
+          <t>AP51</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>MATCH</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP34, Frequency=760, Hop_Value=0x34</t>
+          <t>MISSING_FILE1</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP34, Frequency=760, Hop_Value=0x34</t>
+          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP51, Frequency=782, Hop_Value=0x12</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AP13</t>
+          <t>AP48</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISSING_FILE2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP13, Frequency=788, Hop_Value=0x82</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP13, Frequency=788, Hop_Value=0x82</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP48, Frequency=764, Hop_Value=0xC5</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AP14</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
+          <t>AP42</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP14, Frequency=777, Hop_Value=0xCC</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP42, Frequency=773, Hop_Value=0x5C</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP14, Frequency=777, Hop_Value=0xCC</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP42, Frequency=773, Hop_Value=0x5C</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AP17</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP22</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP17, Frequency=771, Hop_Value=0x65</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP22, Frequency=772, Hop_Value=0x33</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP17, Frequency=771, Hop_Value=0x65</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP22, Frequency=772, Hop_Value=0x34</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AP37</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
+          <t>AP35</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP37, Frequency=773, Hop_Value=0xC3</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP35, Frequency=784, Hop_Value=0x36</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP37, Frequency=773, Hop_Value=0xC3</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP35, Frequency=784, Hop_Value=0x36</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AP42</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
+          <t>AP43</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP42, Frequency=773, Hop_Value=0x5C</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP43, Frequency=777, Hop_Value=0xE8</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP42, Frequency=773, Hop_Value=0x5C</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP43, Frequency=777, Hop_Value=0xE8</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AP7</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP4</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP7, Frequency=767, Hop_Value=0xE9</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP4, Frequency=781, Hop_Value=0xC6</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP7, Frequency=767, Hop_Value=0xE9</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP4, Frequency=781, Hop_Value=0xD1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AP25</t>
-        </is>
-      </c>
-      <c r="B33" s="1" t="inlineStr">
+          <t>AP15</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>MISMATCH</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP25, Frequency=773, Hop_Value=0x62</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP15, Frequency=781, Hop_Value=0x7E</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP25, Frequency=773, Hop_Value=0x61</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP15, Frequency=782, Hop_Value=0x7E</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>frequency_hop_value</t>
+          <t>frequency</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AP21</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
+          <t>AP40</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP21, Frequency=773, Hop_Value=0x2B</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP40, Frequency=763, Hop_Value=0x81</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP21, Frequency=773, Hop_Value=0x2B</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP40, Frequency=763, Hop_Value=0x81</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AP41</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
+          <t>AP13</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP41, Frequency=776, Hop_Value=0xA5</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP13, Frequency=788, Hop_Value=0x82</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP41, Frequency=776, Hop_Value=0xA5</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP13, Frequency=788, Hop_Value=0x82</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AP4</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
+          <t>AP33</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP4, Frequency=781, Hop_Value=0xC6</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP33, Frequency=771, Hop_Value=0xB0</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP4, Frequency=781, Hop_Value=0xC6</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP33, Frequency=771, Hop_Value=0xB0</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AP39</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
+          <t>AP20</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP39, Frequency=767, Hop_Value=0x6A</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP20, Frequency=762, Hop_Value=0xF8</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP39, Frequency=767, Hop_Value=0x6A</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP20, Frequency=762, Hop_Value=0xF8</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AP16</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
+          <t>AP24</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP16, Frequency=787, Hop_Value=0x5B</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP24, Frequency=768, Hop_Value=0xC6</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP16, Frequency=787, Hop_Value=0x5B</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP24, Frequency=768, Hop_Value=0xC6</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AP8</t>
+          <t>AP23</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP8, Frequency=765, Hop_Value=0x82</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP23, Frequency=776, Hop_Value=0xDB</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP8, Frequency=765, Hop_Value=0x83</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>frequency_hop_value</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP23, Frequency=776, Hop_Value=0xDB</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>AP23</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
+          <t>AP30</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP23, Frequency=776, Hop_Value=0xDB</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP30, Frequency=776, Hop_Value=0xA0</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP23, Frequency=776, Hop_Value=0xDB</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP30, Frequency=776, Hop_Value=0xA0</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>AP36</t>
+          <t>AP46</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISSING_FILE2</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP36, Frequency=780, Hop_Value=0x98</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP36, Frequency=780, Hop_Value=0x98</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP46, Frequency=786, Hop_Value=0x79</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>AP1</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
+          <t>AP6</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP1, Frequency=777, Hop_Value=0xE2</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP6, Frequency=784, Hop_Value=0x8E</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP1, Frequency=777, Hop_Value=0xE2</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP6, Frequency=784, Hop_Value=0x8E</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>AP38</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
+          <t>AP25</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP38, Frequency=778, Hop_Value=0x44</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP25, Frequency=773, Hop_Value=0x62</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP38, Frequency=778, Hop_Value=0x44</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP25, Frequency=773, Hop_Value=0x62</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AP40</t>
+          <t>AP55</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>MATCH</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP40, Frequency=763, Hop_Value=0x81</t>
+          <t>MISSING_FILE1</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP40, Frequency=763, Hop_Value=0x81</t>
+          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP55, Frequency=786, Hop_Value=0x9A</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AP31</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
+          <t>AP38</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP31, Frequency=761, Hop_Value=0xA1</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP38, Frequency=778, Hop_Value=0x44</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP31, Frequency=761, Hop_Value=0xA1</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP38, Frequency=778, Hop_Value=0x44</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>AP47</t>
+          <t>AP21</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP47, Frequency=775, Hop_Value=0x1A</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP21, Frequency=773, Hop_Value=0x2B</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP47, Frequency=775, Hop_Value=0x1B</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>frequency_hop_value</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP21, Frequency=773, Hop_Value=0x2B</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>AP33</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP31</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP33, Frequency=771, Hop_Value=0xB0</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP31, Frequency=761, Hop_Value=0xA1</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP33, Frequency=771, Hop_Value=0xB0</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP31, Frequency=761, Hop_Value=0xB1</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>AP20</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
+          <t>AP29</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP20, Frequency=762, Hop_Value=0xF8</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP29, Frequency=776, Hop_Value=0x3A</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP20, Frequency=762, Hop_Value=0xF8</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP29, Frequency=776, Hop_Value=0x3A</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>AP48</t>
+          <t>AP53</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>MATCH</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP48, Frequency=764, Hop_Value=0xC5</t>
+          <t>MISSING_FILE1</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP48, Frequency=764, Hop_Value=0xC5</t>
+          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP53, Frequency=784, Hop_Value=0x56</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>AP43</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
+          <t>AP17</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
         <is>
           <t>MATCH</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP43, Frequency=777, Hop_Value=0xE8</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP17, Frequency=771, Hop_Value=0x65</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP43, Frequency=777, Hop_Value=0xE8</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP17, Frequency=771, Hop_Value=0x65</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>AP27</t>
+          <t>AP49</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>MATCH</t>
+          <t>MISSING_FILE2</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP27, Frequency=762, Hop_Value=0x9E</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP27, Frequency=762, Hop_Value=0x9E</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP49, Frequency=774, Hop_Value=0x3F</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>AP8</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP8, Frequency=765, Hop_Value=0x82</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP8, Frequency=765, Hop_Value=0x82</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>AP34</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP34, Frequency=760, Hop_Value=0x34</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP34, Frequency=760, Hop_Value=0x34</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>AP10</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP10, Frequency=768, Hop_Value=0x17</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP10, Frequency=770, Hop_Value=0x17</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>frequency</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>AP16</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP16, Frequency=787, Hop_Value=0x5B</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP16, Frequency=787, Hop_Value=0x5B</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>AP26</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP26, Frequency=785, Hop_Value=0xBB</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP26, Frequency=786, Hop_Value=0xBB</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>frequency</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Added openpyxl to requirements.txt
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -40,12 +40,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -464,7 +464,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AP36</t>
+          <t>AP13</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr">
@@ -474,217 +474,227 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP36, Frequency=780, Hop_Value=0x98</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP13, Frequency=788, Hop_Value=0x82</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP36, Frequency=780, Hop_Value=0x98</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP13, Frequency=788, Hop_Value=0x82</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AP47</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_FILE2</t>
+          <t>AP1</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP47, Frequency=775, Hop_Value=0x1A</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP1, Frequency=777, Hop_Value=0xE2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP1, Frequency=777, Hop_Value=0xE2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AP1</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP22</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP1, Frequency=777, Hop_Value=0xE2</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP22, Frequency=772, Hop_Value=0x33</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP1, Frequency=777, Hop_Value=0xE2</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP22, Frequency=772, Hop_Value=0x34</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AP50</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_FILE2</t>
+          <t>AP38</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP50, Frequency=763, Hop_Value=0x8C</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP38, Frequency=778, Hop_Value=0x44</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP38, Frequency=778, Hop_Value=0x44</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AP27</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP12</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP27, Frequency=762, Hop_Value=0x9E</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP12, Frequency=784, Hop_Value=0x30</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP27, Frequency=762, Hop_Value=0x9E</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP12, Frequency=784, Hop_Value=0x31</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AP7</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>MISMATCH</t>
+          <t>AP9</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP7, Frequency=767, Hop_Value=0xE9</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP9, Frequency=765, Hop_Value=0x49</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP7, Frequency=767, Hop_Value=0xAA</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>frequency_hop_value</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP9, Frequency=765, Hop_Value=0x49</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AP54</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_FILE1</t>
+          <t>AP20</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP20, Frequency=762, Hop_Value=0xF8</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP54, Frequency=785, Hop_Value=0x78</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP20, Frequency=762, Hop_Value=0xF8</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AP2</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
+          <t>AP30</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>MISMATCH</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP2, Frequency=784, Hop_Value=0x19</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP30, Frequency=776, Hop_Value=0xA1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP2, Frequency=785, Hop_Value=0x19</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP30, Frequency=776, Hop_Value=0xA0</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>frequency</t>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AP44</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>MISMATCH</t>
+          <t>AP6</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP44, Frequency=790, Hop_Value=0x56</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP6, Frequency=784, Hop_Value=0x8E</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP44, Frequency=790, Hop_Value=0x57</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>frequency_hop_value</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP6, Frequency=784, Hop_Value=0x8E</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AP39</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP48</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_FILE2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP39, Frequency=767, Hop_Value=0x6A</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP39, Frequency=767, Hop_Value=0x6A</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP48, Frequency=764, Hop_Value=0xC5</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AP32</t>
+          <t>AP16</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
@@ -694,58 +704,63 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP32, Frequency=769, Hop_Value=0x68</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP16, Frequency=787, Hop_Value=0x5B</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP32, Frequency=769, Hop_Value=0x68</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP16, Frequency=787, Hop_Value=0x5B</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AP52</t>
+          <t>AP7</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>MISSING_FILE1</t>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP7, Frequency=767, Hop_Value=0xE9</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP52, Frequency=783, Hop_Value=0x34</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP7, Frequency=767, Hop_Value=0xAA</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AP14</t>
-        </is>
-      </c>
-      <c r="B14" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP14, Frequency=777, Hop_Value=0xCC</t>
+          <t>AP52</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_FILE1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP14, Frequency=777, Hop_Value=0xCC</t>
+          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP52, Frequency=783, Hop_Value=0x34</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AP19</t>
+          <t>AP35</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
@@ -755,41 +770,46 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP19, Frequency=777, Hop_Value=0xE9</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP35, Frequency=784, Hop_Value=0x36</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP19, Frequency=777, Hop_Value=0xE9</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP35, Frequency=784, Hop_Value=0x36</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AP5</t>
-        </is>
-      </c>
-      <c r="B16" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP18</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP5, Frequency=781, Hop_Value=0x6D</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP18, Frequency=764, Hop_Value=0x1D</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP5, Frequency=781, Hop_Value=0x6D</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP18, Frequency=764, Hop_Value=0x2D</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AP3</t>
+          <t>AP42</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
@@ -799,41 +819,36 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP3, Frequency=774, Hop_Value=0xB7</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP42, Frequency=773, Hop_Value=0x5C</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP3, Frequency=774, Hop_Value=0xB7</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP42, Frequency=773, Hop_Value=0x5C</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AP11</t>
-        </is>
-      </c>
-      <c r="B18" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP46</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_FILE2</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP11, Frequency=766, Hop_Value=0xEF</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP11, Frequency=766, Hop_Value=0xEF</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP46, Frequency=786, Hop_Value=0x79</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AP45</t>
+          <t>AP39</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
@@ -843,34 +858,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP45, Frequency=764, Hop_Value=0xA5</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP39, Frequency=767, Hop_Value=0x6A</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP45, Frequency=764, Hop_Value=0xA5</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP39, Frequency=767, Hop_Value=0x6A</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AP18</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
+          <t>AP31</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>MISMATCH</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP18, Frequency=764, Hop_Value=0x1D</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP31, Frequency=761, Hop_Value=0xA1</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP18, Frequency=764, Hop_Value=0x2D</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP31, Frequency=761, Hop_Value=0xB1</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -882,56 +897,46 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AP12</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>MISMATCH</t>
+          <t>AP34</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP12, Frequency=784, Hop_Value=0x30</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP34, Frequency=760, Hop_Value=0x34</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP12, Frequency=784, Hop_Value=0x31</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>frequency_hop_value</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP34, Frequency=760, Hop_Value=0x34</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AP28</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP28, Frequency=781, Hop_Value=0x46</t>
+          <t>AP51</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_FILE1</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP28, Frequency=781, Hop_Value=0x46</t>
+          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP51, Frequency=782, Hop_Value=0x12</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AP41</t>
+          <t>AP43</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -941,102 +946,117 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP41, Frequency=776, Hop_Value=0xA5</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP43, Frequency=777, Hop_Value=0xE8</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP41, Frequency=776, Hop_Value=0xA5</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP43, Frequency=777, Hop_Value=0xE8</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AP37</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>MISMATCH</t>
+          <t>AP14</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP37, Frequency=773, Hop_Value=0xC3</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP14, Frequency=777, Hop_Value=0xCC</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP37, Frequency=774, Hop_Value=0xC3</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>frequency</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP14, Frequency=777, Hop_Value=0xCC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AP9</t>
-        </is>
-      </c>
-      <c r="B25" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP25</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP9, Frequency=765, Hop_Value=0x49</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP25, Frequency=773, Hop_Value=0x61</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP9, Frequency=765, Hop_Value=0x49</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP25, Frequency=773, Hop_Value=0x62</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AP51</t>
+          <t>AP2</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>MISSING_FILE1</t>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP2, Frequency=784, Hop_Value=0x19</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP51, Frequency=782, Hop_Value=0x12</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP2, Frequency=785, Hop_Value=0x19</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>frequency</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AP48</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_FILE2</t>
+          <t>AP27</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP48, Frequency=764, Hop_Value=0xC5</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP27, Frequency=762, Hop_Value=0x9E</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP27, Frequency=762, Hop_Value=0x9E</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AP42</t>
+          <t>AP24</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
@@ -1046,46 +1066,41 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP42, Frequency=773, Hop_Value=0x5C</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP24, Frequency=768, Hop_Value=0xC6</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP42, Frequency=773, Hop_Value=0x5C</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP24, Frequency=768, Hop_Value=0xC6</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AP22</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>MISMATCH</t>
+          <t>AP21</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP22, Frequency=772, Hop_Value=0x33</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP21, Frequency=773, Hop_Value=0x2B</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP22, Frequency=772, Hop_Value=0x34</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>frequency_hop_value</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP21, Frequency=773, Hop_Value=0x2B</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AP35</t>
+          <t>AP19</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1095,19 +1110,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP35, Frequency=784, Hop_Value=0x36</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP19, Frequency=777, Hop_Value=0xE9</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP35, Frequency=784, Hop_Value=0x36</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP19, Frequency=777, Hop_Value=0xE9</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AP43</t>
+          <t>AP17</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1117,139 +1132,129 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP43, Frequency=777, Hop_Value=0xE8</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP17, Frequency=771, Hop_Value=0x65</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP43, Frequency=777, Hop_Value=0xE8</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP17, Frequency=771, Hop_Value=0x65</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AP4</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
+          <t>AP10</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>MISMATCH</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP4, Frequency=781, Hop_Value=0xC6</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP10, Frequency=768, Hop_Value=0x17</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP4, Frequency=781, Hop_Value=0xD1</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP10, Frequency=770, Hop_Value=0x17</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>frequency_hop_value</t>
+          <t>frequency</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AP15</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>MISMATCH</t>
+          <t>AP45</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP15, Frequency=781, Hop_Value=0x7E</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP45, Frequency=764, Hop_Value=0xA5</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP15, Frequency=782, Hop_Value=0x7E</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>frequency</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP45, Frequency=764, Hop_Value=0xA5</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AP40</t>
-        </is>
-      </c>
-      <c r="B34" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP40, Frequency=763, Hop_Value=0x81</t>
+          <t>AP55</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_FILE1</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP40, Frequency=763, Hop_Value=0x81</t>
+          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP55, Frequency=786, Hop_Value=0x9A</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AP13</t>
-        </is>
-      </c>
-      <c r="B35" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP47</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_FILE2</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP13, Frequency=788, Hop_Value=0x82</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP13, Frequency=788, Hop_Value=0x82</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP47, Frequency=775, Hop_Value=0x1B</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AP33</t>
-        </is>
-      </c>
-      <c r="B36" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP11</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP33, Frequency=771, Hop_Value=0xB0</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP11, Frequency=766, Hop_Value=0xEE</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP33, Frequency=771, Hop_Value=0xB0</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP11, Frequency=766, Hop_Value=0xEF</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AP20</t>
+          <t>AP29</t>
         </is>
       </c>
       <c r="B37" s="1" t="inlineStr">
@@ -1259,41 +1264,46 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP20, Frequency=762, Hop_Value=0xF8</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP29, Frequency=776, Hop_Value=0x3A</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP20, Frequency=762, Hop_Value=0xF8</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP29, Frequency=776, Hop_Value=0x3A</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AP24</t>
-        </is>
-      </c>
-      <c r="B38" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP5</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP24, Frequency=768, Hop_Value=0xC6</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP5, Frequency=780, Hop_Value=0x6D</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP24, Frequency=768, Hop_Value=0xC6</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP5, Frequency=781, Hop_Value=0x6D</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>frequency</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AP23</t>
+          <t>AP36</t>
         </is>
       </c>
       <c r="B39" s="1" t="inlineStr">
@@ -1303,19 +1313,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP23, Frequency=776, Hop_Value=0xDB</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP36, Frequency=780, Hop_Value=0x98</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP23, Frequency=776, Hop_Value=0xDB</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP36, Frequency=780, Hop_Value=0x98</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>AP30</t>
+          <t>AP41</t>
         </is>
       </c>
       <c r="B40" s="1" t="inlineStr">
@@ -1325,119 +1335,139 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP30, Frequency=776, Hop_Value=0xA0</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP41, Frequency=776, Hop_Value=0xA5</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP30, Frequency=776, Hop_Value=0xA0</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP41, Frequency=776, Hop_Value=0xA5</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>AP46</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_FILE2</t>
+          <t>AP28</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP46, Frequency=786, Hop_Value=0x79</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP28, Frequency=781, Hop_Value=0x46</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP28, Frequency=781, Hop_Value=0x46</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>AP6</t>
-        </is>
-      </c>
-      <c r="B42" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP8</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP6, Frequency=784, Hop_Value=0x8E</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP8, Frequency=765, Hop_Value=0x83</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP6, Frequency=784, Hop_Value=0x8E</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP8, Frequency=765, Hop_Value=0x82</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>AP25</t>
-        </is>
-      </c>
-      <c r="B43" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP25, Frequency=773, Hop_Value=0x62</t>
+          <t>AP54</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_FILE1</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP25, Frequency=773, Hop_Value=0x62</t>
+          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP54, Frequency=785, Hop_Value=0x78</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AP55</t>
+          <t>AP4</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>MISSING_FILE1</t>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP4, Frequency=781, Hop_Value=0xC6</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP55, Frequency=786, Hop_Value=0x9A</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP4, Frequency=781, Hop_Value=0xD1</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AP38</t>
-        </is>
-      </c>
-      <c r="B45" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP3</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP38, Frequency=778, Hop_Value=0x44</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP3, Frequency=775, Hop_Value=0xB7</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP38, Frequency=778, Hop_Value=0x44</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP3, Frequency=774, Hop_Value=0xB7</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>frequency</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>AP21</t>
+          <t>AP32</t>
         </is>
       </c>
       <c r="B46" s="1" t="inlineStr">
@@ -1447,85 +1477,85 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP21, Frequency=773, Hop_Value=0x2B</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP32, Frequency=769, Hop_Value=0x68</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP21, Frequency=773, Hop_Value=0x2B</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP32, Frequency=769, Hop_Value=0x68</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>AP31</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>MISMATCH</t>
+          <t>AP23</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP31, Frequency=761, Hop_Value=0xA1</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP23, Frequency=776, Hop_Value=0xDB</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Switch=JT9300L 48 AB, Access_Point=AP31, Frequency=761, Hop_Value=0xB1</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>frequency_hop_value</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP23, Frequency=776, Hop_Value=0xDB</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>AP29</t>
-        </is>
-      </c>
-      <c r="B48" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP49</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_FILE2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP29, Frequency=776, Hop_Value=0x3A</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP29, Frequency=776, Hop_Value=0x3A</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP49, Frequency=774, Hop_Value=0x3F</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>AP53</t>
+          <t>AP44</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>MISSING_FILE1</t>
+          <t>MISMATCH</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP44, Frequency=790, Hop_Value=0x56</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP53, Frequency=784, Hop_Value=0x56</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP44, Frequency=790, Hop_Value=0x57</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>frequency_hop_value</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>AP17</t>
+          <t>AP40</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -1535,58 +1565,58 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP17, Frequency=771, Hop_Value=0x65</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP40, Frequency=763, Hop_Value=0x81</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP17, Frequency=771, Hop_Value=0x65</t>
+          <t>Switch=RT9300L 96 9A, Access_Point=AP40, Frequency=763, Hop_Value=0x81</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>AP49</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_FILE2</t>
+          <t>AP15</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Switch=RT9300L 96 9A, Access_Point=AP49, Frequency=774, Hop_Value=0x3F</t>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP15, Frequency=782, Hop_Value=0x7E</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Switch=JT9300L 48 AB, Access_Point=AP15, Frequency=782, Hop_Value=0x7E</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>AP8</t>
-        </is>
-      </c>
-      <c r="B52" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP8, Frequency=765, Hop_Value=0x82</t>
+          <t>AP53</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_FILE1</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP8, Frequency=765, Hop_Value=0x82</t>
+          <t>Switch=ZX9900Q 77 ZZ, Access_Point=AP53, Frequency=784, Hop_Value=0x56</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>AP34</t>
+          <t>AP33</t>
         </is>
       </c>
       <c r="B53" s="1" t="inlineStr">
@@ -1596,34 +1626,34 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP34, Frequency=760, Hop_Value=0x34</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP33, Frequency=771, Hop_Value=0xB0</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Switch=GT8800X 48 EF, Access_Point=AP34, Frequency=760, Hop_Value=0x34</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP33, Frequency=771, Hop_Value=0xB0</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>AP10</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
+          <t>AP26</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>MISMATCH</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP10, Frequency=768, Hop_Value=0x17</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP26, Frequency=785, Hop_Value=0xBB</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP10, Frequency=770, Hop_Value=0x17</t>
+          <t>Switch=MX7200R 24 GH, Access_Point=AP26, Frequency=786, Hop_Value=0xBB</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -1635,44 +1665,39 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>AP16</t>
-        </is>
-      </c>
-      <c r="B55" s="1" t="inlineStr">
-        <is>
-          <t>MATCH</t>
+          <t>AP50</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>MISSING_FILE2</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP16, Frequency=787, Hop_Value=0x5B</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Switch=NX4500P 24 CD, Access_Point=AP16, Frequency=787, Hop_Value=0x5B</t>
+          <t>Switch=NX4500P 24 CD, Access_Point=AP50, Frequency=763, Hop_Value=0x8C</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>AP26</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
+          <t>AP37</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>MISMATCH</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP26, Frequency=785, Hop_Value=0xBB</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP37, Frequency=773, Hop_Value=0xC3</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Switch=MX7200R 24 GH, Access_Point=AP26, Frequency=786, Hop_Value=0xBB</t>
+          <t>Switch=GT8800X 48 EF, Access_Point=AP37, Frequency=774, Hop_Value=0xC3</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">

</xml_diff>